<commit_message>
Added validatio for part and site sample datasheets
</commit_message>
<xml_diff>
--- a/Copy of TCPL Rulesets - GL1 (1).xlsx
+++ b/Copy of TCPL Rulesets - GL1 (1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SW526XH\Downloads\Data Quality Check\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM-8\Data Rules Set Check\Data_rulesets_check\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA66B17B-FC7B-4105-83D6-ED5D3D08AF72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D9EEC2-96E7-4B82-A2CD-56098E494068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="906" firstSheet="8" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="906" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Availability backup" sheetId="89" state="hidden" r:id="rId1"/>
@@ -59,37 +59,26 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
   <futureMetadata name="XLRICHVALUE" count="2">
     <bk>
       <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+        <ext xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="0"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+        <ext xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="1"/>
         </ext>
       </extLst>
@@ -3548,6 +3537,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3556,9 +3548,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5216,8 +5205,8 @@
     <xdr:to>
       <xdr:col>33</xdr:col>
       <xdr:colOff>131010</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>958900</xdr:rowOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>1721</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5498,9 +5487,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -5538,7 +5527,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -5644,7 +5633,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -5786,7 +5775,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -5810,43 +5799,43 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B2" s="173" t="s">
+      <c r="B2" s="170" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="170" t="s">
+      <c r="C2" s="171" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="173" t="s">
+      <c r="D2" s="170" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="170" t="s">
+      <c r="E2" s="171" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="170" t="s">
+      <c r="F2" s="171" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="170" t="s">
+      <c r="G2" s="171" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="170" t="s">
+      <c r="H2" s="171" t="s">
         <v>6</v>
       </c>
       <c r="I2" s="77"/>
-      <c r="J2" s="172" t="s">
+      <c r="J2" s="173" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="172"/>
-      <c r="L2" s="172"/>
-      <c r="M2" s="172"/>
+      <c r="K2" s="173"/>
+      <c r="L2" s="173"/>
+      <c r="M2" s="173"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B3" s="173"/>
-      <c r="C3" s="171"/>
-      <c r="D3" s="173"/>
-      <c r="E3" s="171"/>
-      <c r="F3" s="171"/>
-      <c r="G3" s="171"/>
-      <c r="H3" s="171"/>
+      <c r="B3" s="170"/>
+      <c r="C3" s="172"/>
+      <c r="D3" s="170"/>
+      <c r="E3" s="172"/>
+      <c r="F3" s="172"/>
+      <c r="G3" s="172"/>
+      <c r="H3" s="172"/>
       <c r="I3" s="78"/>
       <c r="J3" s="4" t="s">
         <v>8</v>
@@ -7143,11 +7132,12 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B26:B31"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="B32:B49"/>
+    <mergeCell ref="C32:C49"/>
+    <mergeCell ref="B50:B61"/>
+    <mergeCell ref="C50:C61"/>
+    <mergeCell ref="B62:B67"/>
+    <mergeCell ref="C62:C67"/>
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="J2:M2"/>
     <mergeCell ref="B4:B11"/>
@@ -7155,12 +7145,11 @@
     <mergeCell ref="B24:B25"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="G2:G3"/>
-    <mergeCell ref="B32:B49"/>
-    <mergeCell ref="C32:C49"/>
-    <mergeCell ref="B50:B61"/>
-    <mergeCell ref="C50:C61"/>
-    <mergeCell ref="B62:B67"/>
-    <mergeCell ref="C62:C67"/>
+    <mergeCell ref="B26:B31"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7196,9 +7185,9 @@
         <v>497</v>
       </c>
       <c r="C2" s="194"/>
-      <c r="D2" s="173"/>
-      <c r="E2" s="173"/>
-      <c r="F2" s="173"/>
+      <c r="D2" s="170"/>
+      <c r="E2" s="170"/>
+      <c r="F2" s="170"/>
     </row>
     <row r="3" spans="1:9" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="51"/>
@@ -7639,7 +7628,7 @@
       <selection activeCell="H4" sqref="H4:J11"/>
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
       <pageSetup orientation="portrait" r:id="rId1"/>
-      <autoFilter ref="A2:O16" xr:uid="{EB4C9DA0-FDC2-40AE-A594-A127AD062A6C}">
+      <autoFilter ref="A2:O16" xr:uid="{F57ADFB0-48CD-4DE6-93CE-19ECA17258C8}">
         <filterColumn colId="11">
           <filters>
             <filter val="No"/>
@@ -7697,9 +7686,9 @@
         <v>549</v>
       </c>
       <c r="C2" s="197"/>
-      <c r="D2" s="172"/>
-      <c r="E2" s="172"/>
-      <c r="F2" s="172"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="173"/>
+      <c r="F2" s="173"/>
     </row>
     <row r="3" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="49"/>
@@ -7934,9 +7923,9 @@
         <v>549</v>
       </c>
       <c r="C2" s="197"/>
-      <c r="D2" s="172"/>
-      <c r="E2" s="172"/>
-      <c r="F2" s="172"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="173"/>
+      <c r="F2" s="173"/>
     </row>
     <row r="3" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="49"/>
@@ -8162,8 +8151,8 @@
         <v>576</v>
       </c>
       <c r="C2" s="205"/>
-      <c r="D2" s="172"/>
-      <c r="E2" s="172"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="173"/>
     </row>
     <row r="3" spans="1:8" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="150"/>
@@ -8178,15 +8167,15 @@
       <c r="E4" s="62"/>
     </row>
     <row r="5" spans="1:8" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="173" t="s">
+      <c r="A5" s="170" t="s">
         <v>577</v>
       </c>
-      <c r="B5" s="173"/>
-      <c r="C5" s="173"/>
-      <c r="D5" s="173"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="173"/>
-      <c r="G5" s="173"/>
+      <c r="B5" s="170"/>
+      <c r="C5" s="170"/>
+      <c r="D5" s="170"/>
+      <c r="E5" s="170"/>
+      <c r="F5" s="170"/>
+      <c r="G5" s="170"/>
       <c r="H5" s="155"/>
     </row>
     <row r="6" spans="1:8" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
@@ -8872,9 +8861,9 @@
         <v>654</v>
       </c>
       <c r="B2" s="206"/>
-      <c r="C2" s="172"/>
-      <c r="D2" s="172"/>
-      <c r="E2" s="172"/>
+      <c r="C2" s="173"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="173"/>
     </row>
     <row r="3" spans="1:7" ht="45.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="27"/>
@@ -8989,9 +8978,9 @@
         <v>658</v>
       </c>
       <c r="B2" s="182"/>
-      <c r="C2" s="172"/>
-      <c r="D2" s="172"/>
-      <c r="E2" s="172"/>
+      <c r="C2" s="173"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="173"/>
     </row>
     <row r="3" spans="1:7" ht="46.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="49"/>
@@ -14602,9 +14591,9 @@
         <v>338</v>
       </c>
       <c r="C2" s="182"/>
-      <c r="D2" s="172"/>
-      <c r="E2" s="172"/>
-      <c r="F2" s="172"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="173"/>
+      <c r="F2" s="173"/>
     </row>
     <row r="3" spans="1:12" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="126"/>
@@ -14868,7 +14857,7 @@
       <selection sqref="A1:K1"/>
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
       <pageSetup orientation="portrait" r:id="rId1"/>
-      <autoFilter ref="A2:P11" xr:uid="{3E3C6FAE-BFA7-47D8-BC74-2983C66C24FC}"/>
+      <autoFilter ref="A2:P11" xr:uid="{7B52993D-1329-40F0-92B9-F6B8DE202BB8}"/>
     </customSheetView>
   </customSheetViews>
   <mergeCells count="5">
@@ -14916,9 +14905,9 @@
         <v>374</v>
       </c>
       <c r="C2" s="188"/>
-      <c r="D2" s="172"/>
-      <c r="E2" s="172"/>
-      <c r="F2" s="172"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="173"/>
+      <c r="F2" s="173"/>
     </row>
     <row r="3" spans="1:9" ht="18.649999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="133"/>
@@ -15730,9 +15719,9 @@
         <v>457</v>
       </c>
       <c r="B2" s="182"/>
-      <c r="C2" s="173"/>
-      <c r="D2" s="173"/>
-      <c r="E2" s="173"/>
+      <c r="C2" s="170"/>
+      <c r="D2" s="170"/>
+      <c r="E2" s="170"/>
     </row>
     <row r="3" spans="1:7" ht="41.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="49"/>
@@ -15927,9 +15916,9 @@
         <v>470</v>
       </c>
       <c r="C2" s="182"/>
-      <c r="D2" s="172"/>
-      <c r="E2" s="172"/>
-      <c r="F2" s="172"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="173"/>
+      <c r="F2" s="173"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="B3" s="49"/>
@@ -16305,18 +16294,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -16338,14 +16327,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE8FBFAC-E23D-4BB4-8CBF-896F42440E38}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF3AF32B-3389-4459-9892-0CB366BDC7B3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -16359,4 +16340,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE8FBFAC-E23D-4BB4-8CBF-896F42440E38}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>